<commit_message>
Add 2026 monthly P&L and GroupRB cost lines to Patriot import
Build a Jan-Sep 2026 P&L (Revenue Detail / Expense Detail / P&L
summary with SUMIFS-driven monthly totals) covering the $99/mo
membership revenue plus GroupRB's Hosting, Seobility, Ubersuggest and
Billing Fee costs for Parts of Practice clients.

Also extend Patriot-Revenue-Import with those same monthly cost
entries as negative same-day-paid transactions alongside the existing
invoice rows.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EWHJ4JSrXozykE2fwAhg1g
</commit_message>
<xml_diff>
--- a/Practice Budget Expenses Revenue Conversion/Patriot-Revenue-Import.xlsx
+++ b/Practice Budget Expenses Revenue Conversion/Patriot-Revenue-Import.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="$#,##0.00;($#,##0.00)"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -425,12 +425,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -453,132 +453,132 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>01/31/2026</t>
+          <t>01/01/2026</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Invoice #22183 - Andy Studer Therapy</t>
+          <t>Billing Fee - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>99</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>01/31/2026</t>
+          <t>01/01/2026</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Invoice #22182 - Gratitude and Growth Counseling LLC</t>
+          <t>Billing Fee - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>99</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>03/02/2026</t>
+          <t>01/01/2026</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Invoice #22188 - Andy Studer Therapy</t>
+          <t>Hosting - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>99</v>
+        <v>-10</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>03/02/2026</t>
+          <t>01/01/2026</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Invoice #22189 - Gratitude and Growth Counseling LLC</t>
+          <t>Hosting - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>99</v>
+        <v>-10</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>03/31/2026</t>
+          <t>01/01/2026</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Invoice #22192 - Andy Studer Therapy</t>
+          <t>Seobility - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>99</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>03/31/2026</t>
+          <t>01/01/2026</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Invoice #22193 - Gratitude and Growth Counseling LLC</t>
+          <t>Seobility - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>99</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>05/04/2026</t>
+          <t>01/01/2026</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Invoice #22197 - Andy Studer Therapy</t>
+          <t>Ubersuggest - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>99</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>05/04/2026</t>
+          <t>01/01/2026</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Invoice #22196 - Gratitude and Growth Counseling LLC</t>
+          <t>Ubersuggest - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>99</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>06/08/2026</t>
+          <t>01/31/2026</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Invoice #22201 - Andy Studer Therapy</t>
+          <t>Invoice #22182 - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C10" s="3" t="n">
@@ -588,12 +588,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>06/08/2026</t>
+          <t>01/31/2026</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Invoice #22202 - Gratitude and Growth Counseling LLC</t>
+          <t>Invoice #22183 - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
@@ -603,76 +603,1186 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>07/01/2026</t>
+          <t>02/01/2026</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Invoice #22206 - Andy Studer Therapy</t>
+          <t>Billing Fee - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>99</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>07/01/2026</t>
+          <t>02/01/2026</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Invoice #22205 - Gratitude and Growth Counseling LLC</t>
+          <t>Billing Fee - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>99</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>08/05/2026</t>
+          <t>02/01/2026</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Invoice #22209 - Andy Studer Therapy</t>
+          <t>Hosting - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>99</v>
+        <v>-10</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>08/05/2026</t>
+          <t>02/01/2026</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Invoice #22210 - Gratitude and Growth Counseling LLC</t>
+          <t>Hosting - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>99</v>
+        <v>-10</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>02/01/2026</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Seobility - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>02/01/2026</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Seobility - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>02/01/2026</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Ubersuggest - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>-6</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>02/01/2026</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Ubersuggest - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>-6</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>03/01/2026</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Billing Fee - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>03/01/2026</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Billing Fee - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>03/01/2026</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Hosting - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>03/01/2026</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Hosting - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>03/01/2026</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Seobility - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>03/01/2026</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Seobility - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>03/01/2026</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Ubersuggest - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>-6</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>03/01/2026</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Ubersuggest - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>-6</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>03/02/2026</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Invoice #22188 - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>03/02/2026</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Invoice #22189 - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>03/31/2026</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Invoice #22192 - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>03/31/2026</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Invoice #22193 - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>04/01/2026</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Billing Fee - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="n">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>04/01/2026</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Billing Fee - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>04/01/2026</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Hosting - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="n">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>04/01/2026</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Hosting - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="n">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>04/01/2026</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Seobility - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="n">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>04/01/2026</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Seobility - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="n">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>04/01/2026</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Ubersuggest - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="n">
+        <v>-6</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>04/01/2026</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Ubersuggest - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="n">
+        <v>-6</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>05/01/2026</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Billing Fee - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="n">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>05/01/2026</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Billing Fee - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="n">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>05/01/2026</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Hosting - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="n">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>05/01/2026</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Hosting - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="n">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>05/01/2026</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Seobility - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="n">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>05/01/2026</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Seobility - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="n">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>05/01/2026</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Ubersuggest - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="n">
+        <v>-6</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>05/01/2026</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Ubersuggest - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="n">
+        <v>-6</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>05/04/2026</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Invoice #22196 - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>05/04/2026</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Invoice #22197 - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>06/01/2026</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Billing Fee - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="n">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>06/01/2026</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Billing Fee - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="n">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>06/01/2026</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Hosting - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="n">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>06/01/2026</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Hosting - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="n">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>06/01/2026</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Seobility - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="n">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>06/01/2026</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Seobility - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="n">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>06/01/2026</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Ubersuggest - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="n">
+        <v>-6</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>06/01/2026</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Ubersuggest - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="n">
+        <v>-6</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>06/08/2026</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Invoice #22201 - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>06/08/2026</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Invoice #22202 - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>07/01/2026</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Billing Fee - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="n">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>07/01/2026</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Billing Fee - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="n">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>07/01/2026</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Hosting - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="n">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>07/01/2026</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Hosting - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="n">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>07/01/2026</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Invoice #22205 - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>07/01/2026</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Invoice #22206 - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>07/01/2026</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Seobility - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="n">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>07/01/2026</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Seobility - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="n">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>07/01/2026</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Ubersuggest - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="n">
+        <v>-6</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>07/01/2026</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Ubersuggest - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="n">
+        <v>-6</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>08/01/2026</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Billing Fee - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="n">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>08/01/2026</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Billing Fee - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="n">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>08/01/2026</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Hosting - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="n">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>08/01/2026</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Hosting - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="n">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>08/01/2026</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Seobility - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="n">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>08/01/2026</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Seobility - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="n">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>08/01/2026</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Ubersuggest - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="n">
+        <v>-6</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>08/01/2026</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Ubersuggest - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="n">
+        <v>-6</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
           <t>08/05/2026</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Invoice #22209 - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Invoice #22210 - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
         <is>
           <t>Invoice #22211 - Guidance Through Grief Counseling Center, PLLC</t>
         </is>
       </c>
-      <c r="C16" s="3" t="n">
+      <c r="C80" s="3" t="n">
         <v>99</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>09/01/2026</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Billing Fee - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="n">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>09/01/2026</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Billing Fee - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="n">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>09/01/2026</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>Billing Fee - Guidance Through Grief Counseling Center, PLLC</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="n">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>09/01/2026</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Hosting - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="n">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>09/01/2026</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>Hosting - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="n">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>09/01/2026</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Hosting - Guidance Through Grief Counseling Center, PLLC</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="n">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>09/01/2026</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>Seobility - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="n">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>09/01/2026</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>Seobility - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="n">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>09/01/2026</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>Ubersuggest - Andy Studer Therapy</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="n">
+        <v>-6</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>09/01/2026</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Ubersuggest - Gratitude and Growth Counseling LLC</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="n">
+        <v>-6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Label Patriot import expense descriptions with GL account names
Prefix each expense transaction's Description with its Patriot GL
account (GroupRB:Hosting, GroupRB:SEO Tools, GroupRB:Bank Fees) so
they can be categorized against those accounts on import, since
Patriot's bank-transaction import format has no separate
account/category field.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EWHJ4JSrXozykE2fwAhg1g
</commit_message>
<xml_diff>
--- a/Practice Budget Expenses Revenue Conversion/Patriot-Revenue-Import.xlsx
+++ b/Practice Budget Expenses Revenue Conversion/Patriot-Revenue-Import.xlsx
@@ -458,7 +458,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Billing Fee - Andy Studer Therapy</t>
+          <t>GroupRB:Bank Fees - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C2" s="3" t="n">
@@ -473,7 +473,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Billing Fee - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:Bank Fees - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
@@ -488,7 +488,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Hosting - Andy Studer Therapy</t>
+          <t>GroupRB:Hosting - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
@@ -503,7 +503,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Hosting - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:Hosting - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
@@ -518,7 +518,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Seobility - Andy Studer Therapy</t>
+          <t>GroupRB:SEO Tools (Seobility) - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Seobility - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:SEO Tools (Seobility) - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
@@ -548,7 +548,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Ubersuggest - Andy Studer Therapy</t>
+          <t>GroupRB:SEO Tools (Ubersuggest) - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C8" s="3" t="n">
@@ -563,7 +563,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Ubersuggest - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:SEO Tools (Ubersuggest) - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Billing Fee - Andy Studer Therapy</t>
+          <t>GroupRB:Bank Fees - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
@@ -623,7 +623,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Billing Fee - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:Bank Fees - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
@@ -638,7 +638,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Hosting - Andy Studer Therapy</t>
+          <t>GroupRB:Hosting - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
@@ -653,7 +653,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Hosting - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:Hosting - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
@@ -668,7 +668,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Seobility - Andy Studer Therapy</t>
+          <t>GroupRB:SEO Tools (Seobility) - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Seobility - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:SEO Tools (Seobility) - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
@@ -698,7 +698,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Ubersuggest - Andy Studer Therapy</t>
+          <t>GroupRB:SEO Tools (Ubersuggest) - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
@@ -713,7 +713,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Ubersuggest - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:SEO Tools (Ubersuggest) - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
@@ -728,7 +728,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Billing Fee - Andy Studer Therapy</t>
+          <t>GroupRB:Bank Fees - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C20" s="3" t="n">
@@ -743,7 +743,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Billing Fee - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:Bank Fees - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C21" s="3" t="n">
@@ -758,7 +758,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Hosting - Andy Studer Therapy</t>
+          <t>GroupRB:Hosting - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C22" s="3" t="n">
@@ -773,7 +773,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Hosting - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:Hosting - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C23" s="3" t="n">
@@ -788,7 +788,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Seobility - Andy Studer Therapy</t>
+          <t>GroupRB:SEO Tools (Seobility) - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C24" s="3" t="n">
@@ -803,7 +803,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Seobility - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:SEO Tools (Seobility) - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C25" s="3" t="n">
@@ -818,7 +818,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Ubersuggest - Andy Studer Therapy</t>
+          <t>GroupRB:SEO Tools (Ubersuggest) - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C26" s="3" t="n">
@@ -833,7 +833,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Ubersuggest - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:SEO Tools (Ubersuggest) - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C27" s="3" t="n">
@@ -908,7 +908,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Billing Fee - Andy Studer Therapy</t>
+          <t>GroupRB:Bank Fees - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C32" s="3" t="n">
@@ -923,7 +923,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Billing Fee - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:Bank Fees - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C33" s="3" t="n">
@@ -938,7 +938,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Hosting - Andy Studer Therapy</t>
+          <t>GroupRB:Hosting - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C34" s="3" t="n">
@@ -953,7 +953,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Hosting - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:Hosting - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C35" s="3" t="n">
@@ -968,7 +968,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Seobility - Andy Studer Therapy</t>
+          <t>GroupRB:SEO Tools (Seobility) - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C36" s="3" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Seobility - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:SEO Tools (Seobility) - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C37" s="3" t="n">
@@ -998,7 +998,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Ubersuggest - Andy Studer Therapy</t>
+          <t>GroupRB:SEO Tools (Ubersuggest) - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C38" s="3" t="n">
@@ -1013,7 +1013,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Ubersuggest - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:SEO Tools (Ubersuggest) - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C39" s="3" t="n">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Billing Fee - Andy Studer Therapy</t>
+          <t>GroupRB:Bank Fees - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C40" s="3" t="n">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Billing Fee - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:Bank Fees - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C41" s="3" t="n">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Hosting - Andy Studer Therapy</t>
+          <t>GroupRB:Hosting - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C42" s="3" t="n">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Hosting - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:Hosting - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C43" s="3" t="n">
@@ -1088,7 +1088,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Seobility - Andy Studer Therapy</t>
+          <t>GroupRB:SEO Tools (Seobility) - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C44" s="3" t="n">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Seobility - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:SEO Tools (Seobility) - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C45" s="3" t="n">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Ubersuggest - Andy Studer Therapy</t>
+          <t>GroupRB:SEO Tools (Ubersuggest) - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C46" s="3" t="n">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Ubersuggest - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:SEO Tools (Ubersuggest) - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C47" s="3" t="n">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Billing Fee - Andy Studer Therapy</t>
+          <t>GroupRB:Bank Fees - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C50" s="3" t="n">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Billing Fee - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:Bank Fees - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C51" s="3" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Hosting - Andy Studer Therapy</t>
+          <t>GroupRB:Hosting - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C52" s="3" t="n">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Hosting - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:Hosting - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C53" s="3" t="n">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Seobility - Andy Studer Therapy</t>
+          <t>GroupRB:SEO Tools (Seobility) - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C54" s="3" t="n">
@@ -1253,7 +1253,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Seobility - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:SEO Tools (Seobility) - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C55" s="3" t="n">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Ubersuggest - Andy Studer Therapy</t>
+          <t>GroupRB:SEO Tools (Ubersuggest) - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C56" s="3" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Ubersuggest - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:SEO Tools (Ubersuggest) - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C57" s="3" t="n">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Billing Fee - Andy Studer Therapy</t>
+          <t>GroupRB:Bank Fees - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C60" s="3" t="n">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Billing Fee - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:Bank Fees - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C61" s="3" t="n">
@@ -1358,7 +1358,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Hosting - Andy Studer Therapy</t>
+          <t>GroupRB:Hosting - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C62" s="3" t="n">
@@ -1373,7 +1373,7 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Hosting - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:Hosting - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C63" s="3" t="n">
@@ -1388,11 +1388,11 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Invoice #22205 - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:SEO Tools (Seobility) - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C64" s="3" t="n">
-        <v>99</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="65">
@@ -1403,11 +1403,11 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Invoice #22206 - Andy Studer Therapy</t>
+          <t>GroupRB:SEO Tools (Seobility) - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C65" s="3" t="n">
-        <v>99</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="66">
@@ -1418,11 +1418,11 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Seobility - Andy Studer Therapy</t>
+          <t>GroupRB:SEO Tools (Ubersuggest) - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C66" s="3" t="n">
-        <v>-5</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="67">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Seobility - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:SEO Tools (Ubersuggest) - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C67" s="3" t="n">
-        <v>-5</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="68">
@@ -1448,11 +1448,11 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Ubersuggest - Andy Studer Therapy</t>
+          <t>Invoice #22205 - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C68" s="3" t="n">
-        <v>-6</v>
+        <v>99</v>
       </c>
     </row>
     <row r="69">
@@ -1463,11 +1463,11 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Ubersuggest - Gratitude and Growth Counseling LLC</t>
+          <t>Invoice #22206 - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C69" s="3" t="n">
-        <v>-6</v>
+        <v>99</v>
       </c>
     </row>
     <row r="70">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Billing Fee - Andy Studer Therapy</t>
+          <t>GroupRB:Bank Fees - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C70" s="3" t="n">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Billing Fee - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:Bank Fees - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C71" s="3" t="n">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Hosting - Andy Studer Therapy</t>
+          <t>GroupRB:Hosting - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C72" s="3" t="n">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>Hosting - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:Hosting - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C73" s="3" t="n">
@@ -1538,7 +1538,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Seobility - Andy Studer Therapy</t>
+          <t>GroupRB:SEO Tools (Seobility) - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C74" s="3" t="n">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>Seobility - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:SEO Tools (Seobility) - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C75" s="3" t="n">
@@ -1568,7 +1568,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Ubersuggest - Andy Studer Therapy</t>
+          <t>GroupRB:SEO Tools (Ubersuggest) - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C76" s="3" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>Ubersuggest - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:SEO Tools (Ubersuggest) - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C77" s="3" t="n">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>Billing Fee - Andy Studer Therapy</t>
+          <t>GroupRB:Bank Fees - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C81" s="3" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Billing Fee - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:Bank Fees - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C82" s="3" t="n">
@@ -1673,7 +1673,7 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>Billing Fee - Guidance Through Grief Counseling Center, PLLC</t>
+          <t>GroupRB:Bank Fees - Guidance Through Grief Counseling Center, PLLC</t>
         </is>
       </c>
       <c r="C83" s="3" t="n">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Hosting - Andy Studer Therapy</t>
+          <t>GroupRB:Hosting - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C84" s="3" t="n">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>Hosting - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:Hosting - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C85" s="3" t="n">
@@ -1718,7 +1718,7 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Hosting - Guidance Through Grief Counseling Center, PLLC</t>
+          <t>GroupRB:Hosting - Guidance Through Grief Counseling Center, PLLC</t>
         </is>
       </c>
       <c r="C86" s="3" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>Seobility - Andy Studer Therapy</t>
+          <t>GroupRB:SEO Tools (Seobility) - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C87" s="3" t="n">
@@ -1748,7 +1748,7 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Seobility - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:SEO Tools (Seobility) - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C88" s="3" t="n">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>Ubersuggest - Andy Studer Therapy</t>
+          <t>GroupRB:SEO Tools (Ubersuggest) - Andy Studer Therapy</t>
         </is>
       </c>
       <c r="C89" s="3" t="n">
@@ -1778,7 +1778,7 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>Ubersuggest - Gratitude and Growth Counseling LLC</t>
+          <t>GroupRB:SEO Tools (Ubersuggest) - Gratitude and Growth Counseling LLC</t>
         </is>
       </c>
       <c r="C90" s="3" t="n">

</xml_diff>